<commit_message>
refactor: update iris.xlsx example data binary file
</commit_message>
<xml_diff>
--- a/app/static/example_data/iris.xlsx
+++ b/app/static/example_data/iris.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meissnerto\Desktop\TexAn2.0\data\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meissnerto\Desktop\TexAn2.0\app\static\example_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DE2EA6-1611-4B92-8E62-68D541DAFF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA700C4-2FDC-4129-B771-B0B86D774097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="1860" windowWidth="38700" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,18 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="8">
   <si>
-    <t>Sepal.Length</t>
-  </si>
-  <si>
-    <t>Sepal.Width</t>
-  </si>
-  <si>
-    <t>Petal.Length</t>
-  </si>
-  <si>
-    <t>Petal.Width</t>
-  </si>
-  <si>
     <t>setosa</t>
   </si>
   <si>
@@ -49,6 +37,18 @@
   </si>
   <si>
     <t>SPECIES</t>
+  </si>
+  <si>
+    <t>SepalLength</t>
+  </si>
+  <si>
+    <t>SepalWidth</t>
+  </si>
+  <si>
+    <t>PetalLength</t>
+  </si>
+  <si>
+    <t>PetalWidth</t>
   </si>
 </sst>
 </file>
@@ -425,19 +425,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -454,7 +454,7 @@
         <v>0.2</v>
       </c>
       <c r="E2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -471,7 +471,7 @@
         <v>0.2</v>
       </c>
       <c r="E3" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -488,7 +488,7 @@
         <v>0.2</v>
       </c>
       <c r="E4" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -505,7 +505,7 @@
         <v>0.2</v>
       </c>
       <c r="E5" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -522,7 +522,7 @@
         <v>0.2</v>
       </c>
       <c r="E6" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -539,7 +539,7 @@
         <v>0.4</v>
       </c>
       <c r="E7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -556,7 +556,7 @@
         <v>0.3</v>
       </c>
       <c r="E8" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -573,7 +573,7 @@
         <v>0.2</v>
       </c>
       <c r="E9" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -590,7 +590,7 @@
         <v>0.2</v>
       </c>
       <c r="E10" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -607,7 +607,7 @@
         <v>0.1</v>
       </c>
       <c r="E11" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -624,7 +624,7 @@
         <v>0.2</v>
       </c>
       <c r="E12" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -641,7 +641,7 @@
         <v>0.2</v>
       </c>
       <c r="E13" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -658,7 +658,7 @@
         <v>0.1</v>
       </c>
       <c r="E14" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -675,7 +675,7 @@
         <v>0.1</v>
       </c>
       <c r="E15" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -692,7 +692,7 @@
         <v>0.2</v>
       </c>
       <c r="E16" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -709,7 +709,7 @@
         <v>0.4</v>
       </c>
       <c r="E17" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -726,7 +726,7 @@
         <v>0.4</v>
       </c>
       <c r="E18" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -743,7 +743,7 @@
         <v>0.3</v>
       </c>
       <c r="E19" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -760,7 +760,7 @@
         <v>0.3</v>
       </c>
       <c r="E20" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -777,7 +777,7 @@
         <v>0.3</v>
       </c>
       <c r="E21" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -794,7 +794,7 @@
         <v>0.2</v>
       </c>
       <c r="E22" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -811,7 +811,7 @@
         <v>0.4</v>
       </c>
       <c r="E23" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -828,7 +828,7 @@
         <v>0.2</v>
       </c>
       <c r="E24" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -845,7 +845,7 @@
         <v>0.5</v>
       </c>
       <c r="E25" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -862,7 +862,7 @@
         <v>0.2</v>
       </c>
       <c r="E26" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -879,7 +879,7 @@
         <v>0.2</v>
       </c>
       <c r="E27" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -896,7 +896,7 @@
         <v>0.4</v>
       </c>
       <c r="E28" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -913,7 +913,7 @@
         <v>0.2</v>
       </c>
       <c r="E29" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -930,7 +930,7 @@
         <v>0.2</v>
       </c>
       <c r="E30" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -947,7 +947,7 @@
         <v>0.2</v>
       </c>
       <c r="E31" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -964,7 +964,7 @@
         <v>0.2</v>
       </c>
       <c r="E32" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -981,7 +981,7 @@
         <v>0.4</v>
       </c>
       <c r="E33" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -998,7 +998,7 @@
         <v>0.1</v>
       </c>
       <c r="E34" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1015,7 +1015,7 @@
         <v>0.2</v>
       </c>
       <c r="E35" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1032,7 +1032,7 @@
         <v>0.2</v>
       </c>
       <c r="E36" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1049,7 +1049,7 @@
         <v>0.2</v>
       </c>
       <c r="E37" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1066,7 +1066,7 @@
         <v>0.2</v>
       </c>
       <c r="E38" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1083,7 +1083,7 @@
         <v>0.1</v>
       </c>
       <c r="E39" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1100,7 +1100,7 @@
         <v>0.2</v>
       </c>
       <c r="E40" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1117,7 +1117,7 @@
         <v>0.2</v>
       </c>
       <c r="E41" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1134,7 +1134,7 @@
         <v>0.3</v>
       </c>
       <c r="E42" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1151,7 +1151,7 @@
         <v>0.3</v>
       </c>
       <c r="E43" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1168,7 +1168,7 @@
         <v>0.2</v>
       </c>
       <c r="E44" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1185,7 +1185,7 @@
         <v>0.6</v>
       </c>
       <c r="E45" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1202,7 +1202,7 @@
         <v>0.4</v>
       </c>
       <c r="E46" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1219,7 +1219,7 @@
         <v>0.3</v>
       </c>
       <c r="E47" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1236,7 +1236,7 @@
         <v>0.2</v>
       </c>
       <c r="E48" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1253,7 +1253,7 @@
         <v>0.2</v>
       </c>
       <c r="E49" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1270,7 +1270,7 @@
         <v>0.2</v>
       </c>
       <c r="E50" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1287,7 +1287,7 @@
         <v>0.2</v>
       </c>
       <c r="E51" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1304,7 +1304,7 @@
         <v>1.4</v>
       </c>
       <c r="E52" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1321,7 +1321,7 @@
         <v>1.5</v>
       </c>
       <c r="E53" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1338,7 +1338,7 @@
         <v>1.5</v>
       </c>
       <c r="E54" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -1355,7 +1355,7 @@
         <v>1.3</v>
       </c>
       <c r="E55" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1372,7 +1372,7 @@
         <v>1.5</v>
       </c>
       <c r="E56" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -1389,7 +1389,7 @@
         <v>1.3</v>
       </c>
       <c r="E57" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -1406,7 +1406,7 @@
         <v>1.6</v>
       </c>
       <c r="E58" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1423,7 +1423,7 @@
         <v>1</v>
       </c>
       <c r="E59" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -1440,7 +1440,7 @@
         <v>1.3</v>
       </c>
       <c r="E60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -1457,7 +1457,7 @@
         <v>1.4</v>
       </c>
       <c r="E61" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -1474,7 +1474,7 @@
         <v>1</v>
       </c>
       <c r="E62" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -1491,7 +1491,7 @@
         <v>1.5</v>
       </c>
       <c r="E63" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -1508,7 +1508,7 @@
         <v>1</v>
       </c>
       <c r="E64" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -1525,7 +1525,7 @@
         <v>1.4</v>
       </c>
       <c r="E65" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -1542,7 +1542,7 @@
         <v>1.3</v>
       </c>
       <c r="E66" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -1559,7 +1559,7 @@
         <v>1.4</v>
       </c>
       <c r="E67" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -1576,7 +1576,7 @@
         <v>1.5</v>
       </c>
       <c r="E68" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -1610,7 +1610,7 @@
         <v>1.5</v>
       </c>
       <c r="E70" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -1627,7 +1627,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="E71" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -1644,7 +1644,7 @@
         <v>1.8</v>
       </c>
       <c r="E72" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -1661,7 +1661,7 @@
         <v>1.3</v>
       </c>
       <c r="E73" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -1678,7 +1678,7 @@
         <v>1.5</v>
       </c>
       <c r="E74" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -1695,7 +1695,7 @@
         <v>1.2</v>
       </c>
       <c r="E75" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -1712,7 +1712,7 @@
         <v>1.3</v>
       </c>
       <c r="E76" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -1729,7 +1729,7 @@
         <v>1.4</v>
       </c>
       <c r="E77" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -1746,7 +1746,7 @@
         <v>1.4</v>
       </c>
       <c r="E78" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -1763,7 +1763,7 @@
         <v>1.7</v>
       </c>
       <c r="E79" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -1780,7 +1780,7 @@
         <v>1.5</v>
       </c>
       <c r="E80" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -1797,7 +1797,7 @@
         <v>1</v>
       </c>
       <c r="E81" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -1814,7 +1814,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="E82" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -1831,7 +1831,7 @@
         <v>1</v>
       </c>
       <c r="E83" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -1848,7 +1848,7 @@
         <v>1.2</v>
       </c>
       <c r="E84" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -1865,7 +1865,7 @@
         <v>1.6</v>
       </c>
       <c r="E85" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -1882,7 +1882,7 @@
         <v>1.5</v>
       </c>
       <c r="E86" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -1899,7 +1899,7 @@
         <v>1.6</v>
       </c>
       <c r="E87" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -1916,7 +1916,7 @@
         <v>1.5</v>
       </c>
       <c r="E88" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -1933,7 +1933,7 @@
         <v>1.3</v>
       </c>
       <c r="E89" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -1950,7 +1950,7 @@
         <v>1.3</v>
       </c>
       <c r="E90" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -1967,7 +1967,7 @@
         <v>1.3</v>
       </c>
       <c r="E91" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -1984,7 +1984,7 @@
         <v>1.2</v>
       </c>
       <c r="E92" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -2001,7 +2001,7 @@
         <v>1.4</v>
       </c>
       <c r="E93" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -2018,7 +2018,7 @@
         <v>1.2</v>
       </c>
       <c r="E94" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -2035,7 +2035,7 @@
         <v>1</v>
       </c>
       <c r="E95" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -2052,7 +2052,7 @@
         <v>1.3</v>
       </c>
       <c r="E96" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2069,7 +2069,7 @@
         <v>1.2</v>
       </c>
       <c r="E97" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2086,7 +2086,7 @@
         <v>1.3</v>
       </c>
       <c r="E98" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2103,7 +2103,7 @@
         <v>1.3</v>
       </c>
       <c r="E99" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2120,7 +2120,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="E100" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2137,7 +2137,7 @@
         <v>1.3</v>
       </c>
       <c r="E101" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2154,7 +2154,7 @@
         <v>2.5</v>
       </c>
       <c r="E102" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2171,7 +2171,7 @@
         <v>1.9</v>
       </c>
       <c r="E103" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2188,7 +2188,7 @@
         <v>2.1</v>
       </c>
       <c r="E104" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2205,7 +2205,7 @@
         <v>1.8</v>
       </c>
       <c r="E105" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2222,7 +2222,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="E106" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2239,7 +2239,7 @@
         <v>2.1</v>
       </c>
       <c r="E107" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2256,7 +2256,7 @@
         <v>1.7</v>
       </c>
       <c r="E108" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2273,7 +2273,7 @@
         <v>1.8</v>
       </c>
       <c r="E109" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2290,7 +2290,7 @@
         <v>1.8</v>
       </c>
       <c r="E110" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2307,7 +2307,7 @@
         <v>2.5</v>
       </c>
       <c r="E111" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2324,7 +2324,7 @@
         <v>2</v>
       </c>
       <c r="E112" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2341,7 +2341,7 @@
         <v>1.9</v>
       </c>
       <c r="E113" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2358,7 +2358,7 @@
         <v>2.1</v>
       </c>
       <c r="E114" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2375,7 +2375,7 @@
         <v>2</v>
       </c>
       <c r="E115" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2392,7 +2392,7 @@
         <v>2.4</v>
       </c>
       <c r="E116" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2409,7 +2409,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E117" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2426,7 +2426,7 @@
         <v>1.8</v>
       </c>
       <c r="E118" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2443,7 +2443,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="E119" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2460,7 +2460,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E120" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2477,7 +2477,7 @@
         <v>1.5</v>
       </c>
       <c r="E121" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2494,7 +2494,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E122" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2511,7 +2511,7 @@
         <v>2</v>
       </c>
       <c r="E123" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2528,7 +2528,7 @@
         <v>2</v>
       </c>
       <c r="E124" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2545,7 +2545,7 @@
         <v>1.8</v>
       </c>
       <c r="E125" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2562,7 +2562,7 @@
         <v>2.1</v>
       </c>
       <c r="E126" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2579,7 +2579,7 @@
         <v>1.8</v>
       </c>
       <c r="E127" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2596,7 +2596,7 @@
         <v>1.8</v>
       </c>
       <c r="E128" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2613,7 +2613,7 @@
         <v>1.8</v>
       </c>
       <c r="E129" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2630,7 +2630,7 @@
         <v>2.1</v>
       </c>
       <c r="E130" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2647,7 +2647,7 @@
         <v>1.6</v>
       </c>
       <c r="E131" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2664,7 +2664,7 @@
         <v>1.9</v>
       </c>
       <c r="E132" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2681,7 +2681,7 @@
         <v>2</v>
       </c>
       <c r="E133" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2698,7 +2698,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="E134" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2715,7 +2715,7 @@
         <v>1.5</v>
       </c>
       <c r="E135" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2732,7 +2732,7 @@
         <v>1.4</v>
       </c>
       <c r="E136" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2749,7 +2749,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E137" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2766,7 +2766,7 @@
         <v>2.4</v>
       </c>
       <c r="E138" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2783,7 +2783,7 @@
         <v>1.8</v>
       </c>
       <c r="E139" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2800,7 +2800,7 @@
         <v>1.8</v>
       </c>
       <c r="E140" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2817,7 +2817,7 @@
         <v>2.1</v>
       </c>
       <c r="E141" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2834,7 +2834,7 @@
         <v>2.4</v>
       </c>
       <c r="E142" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2851,7 +2851,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E143" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2868,7 +2868,7 @@
         <v>1.9</v>
       </c>
       <c r="E144" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2885,7 +2885,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E145" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2902,7 +2902,7 @@
         <v>2.5</v>
       </c>
       <c r="E146" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2919,7 +2919,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E147" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2936,7 +2936,7 @@
         <v>1.9</v>
       </c>
       <c r="E148" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2953,7 +2953,7 @@
         <v>2</v>
       </c>
       <c r="E149" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2970,7 +2970,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E150" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2987,7 +2987,7 @@
         <v>1.8</v>
       </c>
       <c r="E151" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>